<commit_message>
update log with bae ceil gcd DAO
</commit_message>
<xml_diff>
--- a/a_summary_comparison.xlsx
+++ b/a_summary_comparison.xlsx
@@ -23,12 +23,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="382">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="655" uniqueCount="390">
   <si>
     <t xml:space="preserve">Summary Results – total nodes expanded &lt;= C*. Mine are 2 probs avged, others are full avgs</t>
   </si>
   <si>
-    <t xml:space="preserve">BAE*  19-30-57 + 00-49-08 + 03-13-21 + 04-41-10</t>
+    <t xml:space="preserve">BAE*  19-30-57 + 00-49-08 + 03-13-21 + 04-41-10 + 00-44-42</t>
   </si>
   <si>
     <t xml:space="preserve">NBS/NBB WITH NON MONO CLB &lt;C* miscount</t>
@@ -722,6 +722,30 @@
   </si>
   <si>
     <t xml:space="preserve">15 Puzzle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BiDirLBPairs-lb_alter_first_none_bae_a-dirA-selF-ordNONE-verA-dsD-eps1.0-ufFalse-bpmx1False-himpFalse-rustFalse-stF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BiDirLBPairs-lb_alter_first_none_bae_a_eps_ug-dirA-selF-ordNONE-verA-dsD-eps1.0-ufTrue-bpmx1False-himpFalse-rustFalse-stF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BiDirLBPairs-lb_pohl_first_none_bae_a-dirP-selF-ordNONE-verA-dsD-eps1.0-ufFalse-bpmx1False-himpFalse-rustFalse-stF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BiDirLBPairs-lb_pohl_first_none_bae_a_eps_ug-dirP-selF-ordNONE-verA-dsD-eps1.0-ufTrue-bpmx1False-himpFalse-rustFalse-stF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BiDirLBPairs-lb_minb_first_none_bae_a-dirG-selF-ordNONE-verA-dsD-eps1.0-ufFalse-bpmx1False-himpFalse-rustFalse-stF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BiDirLBPairs-lb_minb_first_none_bae_a_eps_ug-dirG-selF-ordNONE-verA-dsD-eps1.0-ufTrue-bpmx1False-himpFalse-rustFalse-stF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BiDirLBPairs-lb_rand_first_none_bae_a-dirR-selF-ordNONE-verA-dsD-eps1.0-ufFalse-bpmx1False-himpFalse-rustFalse-stF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BiDirLBPairs-lb_rand_first_none_bae_a_eps_ug-dirR-selF-ordNONE-verA-dsD-eps1.0-ufTrue-bpmx1False-himpFalse-rustFalse-stF</t>
   </si>
   <si>
     <t xml:space="preserve">BiDirLBPairs-lb_nbs_f_eps-dirNBS-selF-ordNONE-verF-dsP-eps1.0-ufFalse-bpmx1False-himpFalse-rustFalse</t>
@@ -1437,7 +1461,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="52">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1490,11 +1514,11 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="20" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="20" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1583,6 +1607,18 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="21" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="13" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="12" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="14" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2680,40 +2716,56 @@
       <c r="A4" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="V4" s="13"/>
-      <c r="W4" s="14"/>
+      <c r="V4" s="13" t="s">
+        <v>215</v>
+      </c>
+      <c r="W4" s="14" t="s">
+        <v>216</v>
+      </c>
       <c r="X4" s="15"/>
-      <c r="AC4" s="13"/>
-      <c r="AD4" s="13"/>
+      <c r="AC4" s="13" t="s">
+        <v>217</v>
+      </c>
+      <c r="AD4" s="13" t="s">
+        <v>218</v>
+      </c>
       <c r="AE4" s="6"/>
-      <c r="AJ4" s="13"/>
-      <c r="AK4" s="13"/>
-      <c r="AM4" s="13"/>
-      <c r="AN4" s="13"/>
+      <c r="AJ4" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="AK4" s="13" t="s">
+        <v>220</v>
+      </c>
+      <c r="AM4" s="13" t="s">
+        <v>221</v>
+      </c>
+      <c r="AN4" s="13" t="s">
+        <v>222</v>
+      </c>
       <c r="AW4" s="6"/>
       <c r="AX4" s="6" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="BA4" s="6" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="BD4" s="8" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="BE4" s="8"/>
       <c r="BF4" s="6" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="BG4" s="6"/>
       <c r="BH4" s="6" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="BI4" s="6"/>
       <c r="BJ4" s="6" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="BT4" s="6" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="BU4" s="6"/>
       <c r="BV4" s="6" t="s">
@@ -2722,7 +2774,7 @@
       <c r="BW4" s="6"/>
       <c r="BX4" s="6"/>
       <c r="BY4" s="6" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="BZ4" s="6"/>
       <c r="CA4" s="6" t="s">
@@ -2731,11 +2783,11 @@
       <c r="CB4" s="6"/>
       <c r="CC4" s="6"/>
       <c r="CE4" s="6" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="CF4" s="2"/>
       <c r="CL4" s="6" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="CM4" s="6"/>
       <c r="CN4" s="6" t="s">
@@ -2744,7 +2796,7 @@
       <c r="CO4" s="6"/>
       <c r="CP4" s="6"/>
       <c r="CS4" s="6" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="CT4" s="6"/>
       <c r="CU4" s="6" t="s">
@@ -2753,7 +2805,7 @@
       <c r="CV4" s="6"/>
       <c r="CW4" s="6"/>
       <c r="DB4" s="6" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="DC4" s="6"/>
       <c r="DD4" s="6" t="s">
@@ -2762,7 +2814,7 @@
       <c r="DF4" s="6"/>
       <c r="DG4" s="6"/>
       <c r="DI4" s="6" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="DJ4" s="6"/>
       <c r="DK4" s="6" t="s">
@@ -2771,7 +2823,7 @@
       <c r="DL4" s="6"/>
       <c r="DM4" s="6"/>
       <c r="DQ4" s="6" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="DR4" s="6"/>
       <c r="DS4" s="6" t="s">
@@ -2780,7 +2832,7 @@
       <c r="DT4" s="6"/>
       <c r="DU4" s="6"/>
       <c r="DV4" s="6" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="DW4" s="6" t="s">
         <v>210</v>
@@ -2790,7 +2842,7 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="S5" s="16" t="n">
         <v>8039156</v>
@@ -2855,7 +2907,7 @@
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>15549689</v>
@@ -3091,7 +3143,7 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="S7" s="16"/>
       <c r="T7" s="16"/>
@@ -3189,12 +3241,12 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="D10" s="1" t="n">
         <v>57</v>
@@ -3249,10 +3301,10 @@
       </c>
       <c r="U10" s="23"/>
       <c r="V10" s="18" t="n">
-        <v>126.6</v>
+        <v>120.16</v>
       </c>
       <c r="W10" s="18" t="n">
-        <v>172.86</v>
+        <v>172.82</v>
       </c>
       <c r="X10" s="19" t="n">
         <v>172.82</v>
@@ -3270,7 +3322,7 @@
         <v>138.04</v>
       </c>
       <c r="AC10" s="18" t="n">
-        <v>132.18</v>
+        <v>126.38</v>
       </c>
       <c r="AD10" s="18" t="n">
         <v>166.14</v>
@@ -3291,17 +3343,17 @@
         <v>129.5</v>
       </c>
       <c r="AJ10" s="18" t="n">
-        <v>130.32</v>
+        <v>118.9</v>
       </c>
       <c r="AK10" s="18" t="n">
         <v>162.58</v>
       </c>
       <c r="AL10" s="19"/>
       <c r="AM10" s="18" t="n">
-        <v>127.72</v>
+        <v>120.66</v>
       </c>
       <c r="AN10" s="18" t="n">
-        <v>197.3</v>
+        <v>197.26</v>
       </c>
       <c r="AO10" s="19"/>
       <c r="AP10" s="19"/>
@@ -3530,7 +3582,7 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
       <c r="D11" s="1" t="n">
         <v>6416</v>
@@ -3666,7 +3718,7 @@
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="D12" s="1" t="n">
         <v>322099</v>
@@ -3721,10 +3773,10 @@
       </c>
       <c r="U12" s="22"/>
       <c r="V12" s="18" t="n">
-        <v>30192.82</v>
+        <v>12703.84</v>
       </c>
       <c r="W12" s="25" t="n">
-        <v>112115.82</v>
+        <v>113865.02</v>
       </c>
       <c r="X12" s="19" t="n">
         <v>113865.02</v>
@@ -3742,10 +3794,10 @@
         <v>482021.5</v>
       </c>
       <c r="AC12" s="18" t="n">
-        <v>35057.78</v>
+        <v>13292</v>
       </c>
       <c r="AD12" s="18" t="n">
-        <v>91517.54</v>
+        <v>93558.84</v>
       </c>
       <c r="AE12" s="19" t="n">
         <v>93558.84</v>
@@ -3763,17 +3815,17 @@
         <v>264039.92</v>
       </c>
       <c r="AJ12" s="18" t="n">
-        <v>24945.98</v>
+        <v>15190.06</v>
       </c>
       <c r="AK12" s="18" t="n">
-        <v>112344.64</v>
+        <v>112896.06</v>
       </c>
       <c r="AL12" s="19"/>
       <c r="AM12" s="26" t="n">
-        <v>30206.14</v>
+        <v>12862.58</v>
       </c>
       <c r="AN12" s="18" t="n">
-        <v>112140</v>
+        <v>113889.3</v>
       </c>
       <c r="AO12" s="19"/>
       <c r="AP12" s="19"/>
@@ -4132,7 +4184,7 @@
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="S14" s="24"/>
       <c r="T14" s="22"/>
@@ -4312,13 +4364,13 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="DO16" s="2"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="W17" s="19" t="n">
         <v>681523.18</v>
@@ -4520,7 +4572,7 @@
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="D18" s="1" t="n">
         <v>276809</v>
@@ -4575,10 +4627,10 @@
       </c>
       <c r="U18" s="16"/>
       <c r="V18" s="18" t="n">
-        <v>53152.22</v>
+        <v>47959.86</v>
       </c>
       <c r="W18" s="25" t="n">
-        <v>230316.96</v>
+        <v>230315.44</v>
       </c>
       <c r="X18" s="19" t="n">
         <v>230315.44</v>
@@ -4596,10 +4648,10 @@
         <v>245387</v>
       </c>
       <c r="AC18" s="18" t="n">
-        <v>55087.62</v>
+        <v>49513.36</v>
       </c>
       <c r="AD18" s="18" t="n">
-        <v>205326.9</v>
+        <v>205349.16</v>
       </c>
       <c r="AE18" s="19" t="n">
         <v>205349.16</v>
@@ -4617,17 +4669,17 @@
         <v>171804.92</v>
       </c>
       <c r="AJ18" s="18" t="n">
-        <v>60644.34</v>
+        <v>53667.46</v>
       </c>
       <c r="AK18" s="18" t="n">
-        <v>301179.68</v>
+        <v>301179.86</v>
       </c>
       <c r="AL18" s="19"/>
       <c r="AM18" s="26" t="n">
-        <v>53152.6</v>
+        <v>47976.58</v>
       </c>
       <c r="AN18" s="18" t="n">
-        <v>230301.84</v>
+        <v>230301.72</v>
       </c>
       <c r="AO18" s="19"/>
       <c r="AP18" s="19"/>
@@ -4820,7 +4872,7 @@
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
       <c r="D19" s="1" t="n">
         <v>3268093</v>
@@ -4875,10 +4927,10 @@
       </c>
       <c r="U19" s="16"/>
       <c r="V19" s="18" t="n">
-        <v>404342.62</v>
+        <v>385607.16</v>
       </c>
       <c r="W19" s="18" t="n">
-        <v>673927.16</v>
+        <v>673928.18</v>
       </c>
       <c r="X19" s="16"/>
       <c r="Y19" s="16"/>
@@ -4886,10 +4938,10 @@
       <c r="AA19" s="16"/>
       <c r="AB19" s="16"/>
       <c r="AC19" s="18" t="n">
-        <v>405581.92</v>
+        <v>386204.06</v>
       </c>
       <c r="AD19" s="18" t="n">
-        <v>660356.46</v>
+        <v>660351.4</v>
       </c>
       <c r="AE19" s="16"/>
       <c r="AF19" s="16"/>
@@ -4897,17 +4949,17 @@
       <c r="AH19" s="16"/>
       <c r="AI19" s="16"/>
       <c r="AJ19" s="18" t="n">
-        <v>517367.12</v>
+        <v>487770.76</v>
       </c>
       <c r="AK19" s="18" t="n">
         <v>1055189.96</v>
       </c>
       <c r="AL19" s="19"/>
       <c r="AM19" s="18" t="n">
-        <v>404349.82</v>
+        <v>385597.68</v>
       </c>
       <c r="AN19" s="18" t="n">
-        <v>673894.34</v>
+        <v>673895.38</v>
       </c>
       <c r="AO19" s="16"/>
       <c r="AP19" s="16"/>
@@ -5202,7 +5254,7 @@
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="S21" s="16"/>
       <c r="T21" s="16"/>
@@ -5411,7 +5463,7 @@
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
       <c r="S22" s="16"/>
       <c r="T22" s="16"/>
@@ -5623,13 +5675,13 @@
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="DO24" s="2"/>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="B25" s="1" t="n">
         <v>64002</v>
@@ -5690,7 +5742,7 @@
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="DO27" s="2"/>
       <c r="EF27" s="2"/>
@@ -5712,7 +5764,7 @@
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="B28" s="1" t="n">
         <v>9646</v>
@@ -5773,10 +5825,10 @@
       </c>
       <c r="U28" s="16"/>
       <c r="V28" s="18" t="n">
-        <v>6336.70974912671</v>
+        <v>6332.17021276596</v>
       </c>
       <c r="W28" s="25" t="n">
-        <v>7027.14226738647</v>
+        <v>7026.72626230549</v>
       </c>
       <c r="X28" s="16"/>
       <c r="Y28" s="16"/>
@@ -5784,10 +5836,10 @@
       <c r="AA28" s="16"/>
       <c r="AB28" s="16"/>
       <c r="AC28" s="18" t="n">
-        <v>5855.38361384567</v>
+        <v>5845.72785011115</v>
       </c>
       <c r="AD28" s="18" t="n">
-        <v>6922.18069228327</v>
+        <v>6925.23245474754</v>
       </c>
       <c r="AE28" s="16"/>
       <c r="AF28" s="16"/>
@@ -5795,17 +5847,17 @@
       <c r="AH28" s="16"/>
       <c r="AI28" s="16"/>
       <c r="AJ28" s="18" t="n">
-        <v>7327.55319148936</v>
+        <v>7319.51413147031</v>
       </c>
       <c r="AK28" s="18" t="n">
-        <v>7982.49761829152</v>
+        <v>7982.48936170213</v>
       </c>
       <c r="AL28" s="19"/>
       <c r="AM28" s="26" t="n">
-        <v>6338.24896792633</v>
+        <v>6334.43251825977</v>
       </c>
       <c r="AN28" s="18" t="n">
-        <v>7030.54906319467</v>
+        <v>7030.04255319149</v>
       </c>
       <c r="AO28" s="16"/>
       <c r="AP28" s="16"/>
@@ -5953,7 +6005,7 @@
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="S29" s="16"/>
       <c r="T29" s="16"/>
@@ -6006,7 +6058,7 @@
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="E31" s="1" t="n">
         <f aca="false">AVERAGE(E10,E12,E18,E19,E28)</f>
@@ -6092,7 +6144,7 @@
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="O32" s="1" t="n">
         <f aca="false">AVERAGE(O6,O10,O12,O18,O19,O28,)</f>
@@ -6150,7 +6202,7 @@
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O37" s="1" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="DO37" s="2"/>
     </row>
@@ -6168,7 +6220,7 @@
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
@@ -6195,7 +6247,7 @@
         <v>115</v>
       </c>
       <c r="R43" s="2" t="s">
-        <v>252</v>
+        <v>260</v>
       </c>
       <c r="S43" s="5" t="s">
         <v>117</v>
@@ -6241,7 +6293,7 @@
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
@@ -6288,7 +6340,7 @@
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="H45" s="19"/>
       <c r="I45" s="2"/>
@@ -6490,7 +6542,7 @@
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="H46" s="19"/>
       <c r="I46" s="2"/>
@@ -6594,14 +6646,14 @@
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
       <c r="H48" s="2"/>
       <c r="DO48" s="2"/>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="I49" s="19"/>
       <c r="O49" s="1" t="n">
@@ -6624,7 +6676,7 @@
       </c>
       <c r="U49" s="23"/>
       <c r="V49" s="18" t="n">
-        <v>77.42</v>
+        <v>71.14</v>
       </c>
       <c r="W49" s="18" t="n">
         <v>66.72</v>
@@ -6645,7 +6697,7 @@
         <v>117.9</v>
       </c>
       <c r="AC49" s="18" t="n">
-        <v>77.22</v>
+        <v>73.18</v>
       </c>
       <c r="AD49" s="18" t="n">
         <v>72.02</v>
@@ -6666,14 +6718,14 @@
         <v>106.02</v>
       </c>
       <c r="AJ49" s="18" t="n">
-        <v>82.84</v>
+        <v>71.86</v>
       </c>
       <c r="AK49" s="18" t="n">
         <v>69.42</v>
       </c>
       <c r="AL49" s="31"/>
       <c r="AM49" s="18" t="n">
-        <v>75.2</v>
+        <v>68.56</v>
       </c>
       <c r="AN49" s="18" t="n">
         <v>64.5</v>
@@ -6907,7 +6959,7 @@
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
       <c r="J50" s="19"/>
       <c r="K50" s="19"/>
@@ -7015,7 +7067,7 @@
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="J51" s="19"/>
       <c r="K51" s="19"/>
@@ -7039,10 +7091,10 @@
       </c>
       <c r="U51" s="33"/>
       <c r="V51" s="18" t="n">
-        <v>29510.54</v>
+        <v>11251.46</v>
       </c>
       <c r="W51" s="25" t="n">
-        <v>111887.32</v>
+        <v>102423.3</v>
       </c>
       <c r="X51" s="19" t="n">
         <v>102423.3</v>
@@ -7060,10 +7112,10 @@
         <v>482021.5</v>
       </c>
       <c r="AC51" s="18" t="n">
-        <v>34384.4</v>
+        <v>11824</v>
       </c>
       <c r="AD51" s="18" t="n">
-        <v>91305.22</v>
+        <v>83188.4</v>
       </c>
       <c r="AE51" s="19" t="n">
         <v>83188.4</v>
@@ -7081,17 +7133,17 @@
         <v>264039.92</v>
       </c>
       <c r="AJ51" s="18" t="n">
-        <v>24232.16</v>
+        <v>11851.5</v>
       </c>
       <c r="AK51" s="18" t="n">
-        <v>110720.1</v>
+        <v>97731.44</v>
       </c>
       <c r="AL51" s="19"/>
       <c r="AM51" s="26" t="n">
-        <v>29516.44</v>
+        <v>11256.6</v>
       </c>
       <c r="AN51" s="18" t="n">
-        <v>111913.54</v>
+        <v>102434.46</v>
       </c>
       <c r="AO51" s="19"/>
       <c r="AP51" s="19"/>
@@ -7454,7 +7506,7 @@
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="J53" s="19"/>
       <c r="K53" s="19"/>
@@ -7637,12 +7689,12 @@
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="W56" s="19" t="n">
         <v>679627.42</v>
@@ -7846,7 +7898,7 @@
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="O57" s="1" t="n">
         <v>276000</v>
@@ -7868,10 +7920,10 @@
       </c>
       <c r="U57" s="29"/>
       <c r="V57" s="18" t="n">
-        <v>52056.16</v>
+        <v>46214.54</v>
       </c>
       <c r="W57" s="25" t="n">
-        <v>217132.48</v>
+        <v>211116.12</v>
       </c>
       <c r="X57" s="31" t="n">
         <v>211116.12</v>
@@ -7889,10 +7941,10 @@
         <v>245387</v>
       </c>
       <c r="AC57" s="18" t="n">
-        <v>53562.64</v>
+        <v>47227.2</v>
       </c>
       <c r="AD57" s="18" t="n">
-        <v>191558.54</v>
+        <v>178701.94</v>
       </c>
       <c r="AE57" s="31" t="n">
         <v>178701.94</v>
@@ -7910,17 +7962,17 @@
         <v>171804.92</v>
       </c>
       <c r="AJ57" s="18" t="n">
-        <v>60603.54</v>
+        <v>53628.1</v>
       </c>
       <c r="AK57" s="18" t="n">
-        <v>300899.02</v>
+        <v>300887.06</v>
       </c>
       <c r="AL57" s="31"/>
       <c r="AM57" s="26" t="n">
-        <v>52061.68</v>
+        <v>46194.9</v>
       </c>
       <c r="AN57" s="18" t="n">
-        <v>217131.68</v>
+        <v>211087.8</v>
       </c>
       <c r="AO57" s="31"/>
       <c r="AP57" s="31"/>
@@ -8111,7 +8163,7 @@
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
       <c r="J58" s="19"/>
       <c r="K58" s="19"/>
@@ -8135,10 +8187,10 @@
       </c>
       <c r="U58" s="29"/>
       <c r="V58" s="18" t="n">
-        <v>402849.6</v>
+        <v>381511.72</v>
       </c>
       <c r="W58" s="18" t="n">
-        <v>667610</v>
+        <v>632674.78</v>
       </c>
       <c r="X58" s="29"/>
       <c r="Y58" s="29"/>
@@ -8146,10 +8198,10 @@
       <c r="AA58" s="29"/>
       <c r="AB58" s="29"/>
       <c r="AC58" s="18" t="n">
-        <v>405216.62</v>
+        <v>381994.78</v>
       </c>
       <c r="AD58" s="18" t="n">
-        <v>651691.62</v>
+        <v>623247.36</v>
       </c>
       <c r="AE58" s="29"/>
       <c r="AF58" s="29"/>
@@ -8157,17 +8209,17 @@
       <c r="AH58" s="29"/>
       <c r="AI58" s="29"/>
       <c r="AJ58" s="18" t="n">
-        <v>516330.02</v>
+        <v>481831.3</v>
       </c>
       <c r="AK58" s="18" t="n">
-        <v>1042770.98</v>
+        <v>974263.44</v>
       </c>
       <c r="AL58" s="19"/>
       <c r="AM58" s="18" t="n">
-        <v>402856.26</v>
+        <v>381480.42</v>
       </c>
       <c r="AN58" s="18" t="n">
-        <v>667610.94</v>
+        <v>632692.34</v>
       </c>
       <c r="AO58" s="29"/>
       <c r="AP58" s="29"/>
@@ -8462,7 +8514,7 @@
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="J60" s="19"/>
       <c r="K60" s="19"/>
@@ -8672,7 +8724,7 @@
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
       <c r="J61" s="19"/>
       <c r="K61" s="19"/>
@@ -8886,17 +8938,17 @@
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="BL66" s="2"/>
       <c r="EF66" s="19"/>
@@ -8917,7 +8969,7 @@
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="O67" s="1" t="n">
         <v>5322</v>
@@ -8938,40 +8990,40 @@
         <v>5246.35535090505</v>
       </c>
       <c r="U67" s="29"/>
-      <c r="V67" s="18" t="n">
-        <v>6060.49825341378</v>
-      </c>
-      <c r="W67" s="25" t="n">
-        <v>6719.3007303906</v>
+      <c r="V67" s="37" t="n">
+        <v>6052.80882819943</v>
+      </c>
+      <c r="W67" s="38" t="n">
+        <v>6694.84153699587</v>
       </c>
       <c r="X67" s="29"/>
       <c r="Y67" s="29"/>
       <c r="Z67" s="29"/>
       <c r="AA67" s="29"/>
       <c r="AB67" s="29"/>
-      <c r="AC67" s="18" t="n">
-        <v>5406.64337885043</v>
-      </c>
-      <c r="AD67" s="18" t="n">
-        <v>6254.71641791045</v>
+      <c r="AC67" s="37" t="n">
+        <v>5396.07780247698</v>
+      </c>
+      <c r="AD67" s="37" t="n">
+        <v>6231.3912353128</v>
       </c>
       <c r="AE67" s="29"/>
       <c r="AF67" s="29"/>
       <c r="AG67" s="29"/>
       <c r="AH67" s="29"/>
       <c r="AI67" s="29"/>
-      <c r="AJ67" s="18" t="n">
-        <v>7172.66084471261</v>
-      </c>
-      <c r="AK67" s="18" t="n">
-        <v>7814.77675452525</v>
+      <c r="AJ67" s="37" t="n">
+        <v>7161.19307716736</v>
+      </c>
+      <c r="AK67" s="37" t="n">
+        <v>7798.87869164814</v>
       </c>
       <c r="AL67" s="19"/>
-      <c r="AM67" s="26" t="n">
-        <v>6062.03207367418</v>
-      </c>
-      <c r="AN67" s="18" t="n">
-        <v>6721.81454429978</v>
+      <c r="AM67" s="39" t="n">
+        <v>6054.6951413147</v>
+      </c>
+      <c r="AN67" s="37" t="n">
+        <v>6697.53413782153</v>
       </c>
       <c r="AO67" s="29"/>
       <c r="AP67" s="29"/>
@@ -9103,7 +9155,7 @@
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="S68" s="29"/>
       <c r="T68" s="29"/>
@@ -9141,7 +9193,7 @@
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="1" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="O70" s="1" t="n">
         <f aca="false">AVERAGE(O49,O51,O57,O58,O67)</f>
@@ -9182,7 +9234,7 @@
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="1" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="O71" s="1" t="n">
         <f aca="false">AVERAGE(O45,O49,O51,O57,O58,O67,)</f>
@@ -9287,13 +9339,13 @@
         <v>138</v>
       </c>
       <c r="AS86" s="1" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
       <c r="AT86" s="1" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
       <c r="AU86" s="1" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="AX86" s="2"/>
       <c r="AY86" s="2"/>
@@ -9381,7 +9433,7 @@
         <v>19</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9403,7 +9455,7 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>258</v>
+        <v>266</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9413,26 +9465,26 @@
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>259</v>
-      </c>
-      <c r="C7" s="37" t="n">
+        <v>267</v>
+      </c>
+      <c r="C7" s="40" t="n">
         <v>684.052721581459</v>
       </c>
-      <c r="D7" s="37" t="n">
+      <c r="D7" s="40" t="n">
         <v>712.43826887846</v>
       </c>
-      <c r="E7" s="38" t="n">
+      <c r="E7" s="41" t="n">
         <v>676.54386572361</v>
       </c>
-      <c r="F7" s="37" t="n">
+      <c r="F7" s="40" t="n">
         <v>790.856329123974</v>
       </c>
-      <c r="G7" s="37" t="n">
+      <c r="G7" s="40" t="n">
         <v>714.333313083649</v>
       </c>
     </row>
@@ -9441,30 +9493,30 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="C12" s="39" t="n">
+        <v>243</v>
+      </c>
+      <c r="C12" s="42" t="n">
         <v>34.1211344003677</v>
       </c>
-      <c r="D12" s="40" t="n">
+      <c r="D12" s="43" t="n">
         <v>13.4298436546326</v>
       </c>
-      <c r="E12" s="39" t="n">
+      <c r="E12" s="42" t="n">
         <v>14.6293577003479</v>
       </c>
       <c r="F12" s="24" t="n">
@@ -9479,22 +9531,22 @@
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9502,12 +9554,12 @@
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9515,12 +9567,12 @@
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9528,17 +9580,17 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9548,26 +9600,26 @@
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>259</v>
-      </c>
-      <c r="C32" s="38" t="n">
+        <v>267</v>
+      </c>
+      <c r="C32" s="41" t="n">
         <v>24529.6949119625</v>
       </c>
-      <c r="D32" s="37" t="n">
+      <c r="D32" s="40" t="n">
         <v>19578.1430439508</v>
       </c>
-      <c r="E32" s="41" t="n">
+      <c r="E32" s="44" t="n">
         <v>19049.1565588771</v>
       </c>
-      <c r="F32" s="37" t="n">
+      <c r="F32" s="40" t="n">
         <v>18584.7486364329</v>
       </c>
-      <c r="G32" s="37" t="n">
+      <c r="G32" s="40" t="n">
         <v>18216.3597551661</v>
       </c>
     </row>
@@ -9576,30 +9628,30 @@
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="C37" s="40" t="n">
+        <v>243</v>
+      </c>
+      <c r="C37" s="43" t="n">
         <v>10586.6811481229</v>
       </c>
-      <c r="D37" s="39" t="n">
+      <c r="D37" s="42" t="n">
         <v>8940.85410665637</v>
       </c>
-      <c r="E37" s="39" t="n">
+      <c r="E37" s="42" t="n">
         <v>8252.47786874597</v>
       </c>
       <c r="F37" s="24" t="n">
@@ -9614,22 +9666,22 @@
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9637,12 +9689,12 @@
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9650,12 +9702,12 @@
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9663,17 +9715,17 @@
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9683,26 +9735,26 @@
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>259</v>
-      </c>
-      <c r="C57" s="42" t="n">
+        <v>267</v>
+      </c>
+      <c r="C57" s="45" t="n">
         <v>241.46</v>
       </c>
-      <c r="D57" s="42" t="n">
+      <c r="D57" s="45" t="n">
         <v>240.09</v>
       </c>
-      <c r="E57" s="43" t="n">
+      <c r="E57" s="46" t="n">
         <v>77.49</v>
       </c>
-      <c r="F57" s="42" t="n">
+      <c r="F57" s="45" t="n">
         <v>226.34</v>
       </c>
-      <c r="G57" s="42" t="n">
+      <c r="G57" s="45" t="n">
         <v>204.92</v>
       </c>
     </row>
@@ -9711,30 +9763,30 @@
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="C62" s="44" t="n">
+        <v>243</v>
+      </c>
+      <c r="C62" s="47" t="n">
         <v>4.21</v>
       </c>
-      <c r="D62" s="45" t="n">
+      <c r="D62" s="48" t="n">
         <v>1.65</v>
       </c>
-      <c r="E62" s="44" t="n">
+      <c r="E62" s="47" t="n">
         <v>2.11</v>
       </c>
       <c r="F62" s="36" t="n">
@@ -9749,22 +9801,22 @@
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9772,12 +9824,12 @@
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="1" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="1" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9785,12 +9837,12 @@
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="1" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9798,12 +9850,12 @@
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="1" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="1" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
     </row>
   </sheetData>
@@ -9891,64 +9943,64 @@
         <v>0</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
       <c r="T1" s="2"/>
       <c r="U1" s="2"/>
       <c r="V1" s="2"/>
       <c r="AF1" s="1" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="AG1" s="1" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="AH1" s="1" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="AJ1" s="1" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="AN1" s="1" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="AO1" s="1" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="AP1" s="1" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="AQ1" s="1" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="AR1" s="1" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="AS1" s="1" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="AU1" s="1" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="AV1" s="1" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="AW1" s="1" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="AY1" s="1" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="BA1" s="1" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="BC1" s="1" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="BL1" s="1" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
       <c r="BN1" s="1" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9971,55 +10023,55 @@
         <v>40</v>
       </c>
       <c r="AF2" s="4" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
       <c r="AG2" s="4" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
       <c r="AH2" s="4" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="AJ2" s="4" t="s">
-        <v>271</v>
+        <v>279</v>
       </c>
       <c r="AN2" s="4" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
       <c r="AO2" s="4" t="s">
-        <v>273</v>
+        <v>281</v>
       </c>
       <c r="AP2" s="4" t="s">
-        <v>274</v>
+        <v>282</v>
       </c>
       <c r="AQ2" s="4" t="s">
         <v>51</v>
       </c>
       <c r="AR2" s="4" t="s">
-        <v>275</v>
+        <v>283</v>
       </c>
       <c r="AS2" s="4" t="s">
-        <v>276</v>
+        <v>284</v>
       </c>
       <c r="AU2" s="4" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
       <c r="AV2" s="4" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
       <c r="AW2" s="4" t="s">
-        <v>279</v>
+        <v>287</v>
       </c>
       <c r="AY2" s="4" t="s">
-        <v>280</v>
+        <v>288</v>
       </c>
       <c r="BA2" s="4" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="BE2" s="4" t="s">
-        <v>282</v>
+        <v>290</v>
       </c>
       <c r="BL2" s="1" t="s">
-        <v>283</v>
+        <v>291</v>
       </c>
       <c r="BO2" s="1" t="s">
         <v>115</v>
@@ -10075,13 +10127,13 @@
         <v>115</v>
       </c>
       <c r="R3" s="1" t="s">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="S3" s="1" t="s">
-        <v>285</v>
+        <v>293</v>
       </c>
       <c r="T3" s="7" t="s">
-        <v>286</v>
+        <v>294</v>
       </c>
       <c r="U3" s="5" t="s">
         <v>117</v>
@@ -10090,10 +10142,10 @@
         <v>118</v>
       </c>
       <c r="W3" s="1" t="s">
-        <v>287</v>
+        <v>295</v>
       </c>
       <c r="X3" s="1" t="s">
-        <v>288</v>
+        <v>296</v>
       </c>
       <c r="AA3" s="4" t="s">
         <v>138</v>
@@ -10108,67 +10160,67 @@
         <v>141</v>
       </c>
       <c r="AF3" s="8" t="s">
-        <v>289</v>
+        <v>297</v>
       </c>
       <c r="AG3" s="8" t="s">
-        <v>290</v>
+        <v>298</v>
       </c>
       <c r="AH3" s="8" t="s">
-        <v>291</v>
+        <v>299</v>
       </c>
       <c r="AJ3" s="8" t="s">
-        <v>292</v>
+        <v>300</v>
       </c>
       <c r="AK3" s="7" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="AL3" s="7" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
       <c r="AM3" s="7" t="s">
-        <v>295</v>
+        <v>303</v>
       </c>
       <c r="AN3" s="8" t="s">
-        <v>296</v>
+        <v>304</v>
       </c>
       <c r="AO3" s="8" t="s">
-        <v>297</v>
+        <v>305</v>
       </c>
       <c r="AP3" s="8" t="s">
-        <v>298</v>
+        <v>306</v>
       </c>
       <c r="AQ3" s="8" t="s">
-        <v>299</v>
+        <v>307</v>
       </c>
       <c r="AR3" s="8" t="s">
-        <v>300</v>
+        <v>308</v>
       </c>
       <c r="AS3" s="8" t="s">
-        <v>301</v>
+        <v>309</v>
       </c>
       <c r="AU3" s="8" t="s">
-        <v>302</v>
+        <v>310</v>
       </c>
       <c r="AV3" s="8" t="s">
-        <v>303</v>
+        <v>311</v>
       </c>
       <c r="AW3" s="7" t="s">
         <v>196</v>
       </c>
       <c r="AY3" s="7" t="s">
-        <v>304</v>
+        <v>312</v>
       </c>
       <c r="BA3" s="10" t="s">
-        <v>305</v>
+        <v>313</v>
       </c>
       <c r="BB3" s="8" t="s">
-        <v>306</v>
+        <v>314</v>
       </c>
       <c r="BC3" s="8" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="BD3" s="8" t="s">
-        <v>308</v>
+        <v>316</v>
       </c>
       <c r="BE3" s="8" t="s">
         <v>155</v>
@@ -10180,28 +10232,28 @@
         <v>160</v>
       </c>
       <c r="BH3" s="8" t="s">
-        <v>309</v>
+        <v>317</v>
       </c>
       <c r="BI3" s="8" t="s">
         <v>191</v>
       </c>
       <c r="BJ3" s="8" t="s">
-        <v>310</v>
+        <v>318</v>
       </c>
       <c r="BL3" s="10" t="s">
-        <v>311</v>
+        <v>319</v>
       </c>
       <c r="BM3" s="8" t="s">
         <v>189</v>
       </c>
       <c r="BN3" s="8" t="s">
-        <v>312</v>
+        <v>320</v>
       </c>
       <c r="BO3" s="8" t="s">
         <v>172</v>
       </c>
       <c r="BP3" s="8" t="s">
-        <v>313</v>
+        <v>321</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10211,7 +10263,7 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="R5" s="17" t="n">
         <v>8060452.5</v>
@@ -10248,7 +10300,7 @@
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>15549689</v>
@@ -10410,12 +10462,12 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="D9" s="1" t="n">
         <v>57</v>
@@ -10593,7 +10645,7 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
       <c r="D10" s="1" t="n">
         <v>6416</v>
@@ -10682,7 +10734,7 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="D11" s="1" t="n">
         <v>322099</v>
@@ -10860,17 +10912,17 @@
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="D15" s="1" t="n">
         <v>276809</v>
@@ -10929,7 +10981,7 @@
       <c r="V15" s="16" t="n">
         <v>276087.16</v>
       </c>
-      <c r="W15" s="46" t="n">
+      <c r="W15" s="49" t="n">
         <v>564610.52</v>
       </c>
       <c r="X15" s="16" t="n">
@@ -10955,7 +11007,7 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
       <c r="D16" s="1" t="n">
         <v>3268093</v>
@@ -11014,7 +11066,7 @@
       <c r="V16" s="16" t="n">
         <v>3265722.1</v>
       </c>
-      <c r="W16" s="47" t="n">
+      <c r="W16" s="50" t="n">
         <v>3674516.76</v>
       </c>
       <c r="X16" s="17" t="n">
@@ -11040,12 +11092,12 @@
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>64002</v>
@@ -11086,7 +11138,7 @@
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="BA21" s="2"/>
       <c r="BB21" s="2"/>
@@ -11107,7 +11159,7 @@
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>9646</v>
@@ -11280,7 +11332,7 @@
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="E24" s="1" t="n">
         <f aca="false">AVERAGE(E9,E11,E15,E16,E22)</f>
@@ -11381,7 +11433,7 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="O25" s="1" t="n">
         <f aca="false">AVERAGE(O6,O9,O11,O15,O16,O22,)</f>
@@ -11422,27 +11474,27 @@
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="T26" s="1" t="s">
-        <v>314</v>
+        <v>322</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="T27" s="1" t="s">
-        <v>315</v>
+        <v>323</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O30" s="1" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="T33" s="1" t="s">
-        <v>316</v>
+        <v>324</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
@@ -11451,7 +11503,7 @@
         <v>18</v>
       </c>
       <c r="R35" s="1" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
       <c r="AY35" s="2"/>
     </row>
@@ -11472,13 +11524,13 @@
         <v>115</v>
       </c>
       <c r="R36" s="1" t="s">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="S36" s="1" t="s">
-        <v>285</v>
+        <v>293</v>
       </c>
       <c r="T36" s="1" t="s">
-        <v>286</v>
+        <v>294</v>
       </c>
       <c r="U36" s="5" t="s">
         <v>117</v>
@@ -11487,10 +11539,10 @@
         <v>118</v>
       </c>
       <c r="W36" s="1" t="s">
-        <v>287</v>
+        <v>295</v>
       </c>
       <c r="X36" s="1" t="s">
-        <v>288</v>
+        <v>296</v>
       </c>
       <c r="AA36" s="1" t="s">
         <v>138</v>
@@ -11507,7 +11559,7 @@
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
@@ -11547,7 +11599,7 @@
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="H38" s="19"/>
       <c r="I38" s="2"/>
@@ -11678,13 +11730,13 @@
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
       <c r="H40" s="2"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="I41" s="19"/>
       <c r="O41" s="1" t="n">
@@ -11830,7 +11882,7 @@
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
       <c r="J42" s="19"/>
       <c r="K42" s="19"/>
@@ -11891,7 +11943,7 @@
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="J43" s="19"/>
       <c r="K43" s="19"/>
@@ -12042,17 +12094,17 @@
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="O47" s="1" t="n">
         <v>276000</v>
@@ -12101,7 +12153,7 @@
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
       <c r="J48" s="19"/>
       <c r="K48" s="19"/>
@@ -12157,17 +12209,17 @@
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="AO53" s="2"/>
       <c r="AP53" s="2"/>
@@ -12200,7 +12252,7 @@
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="O54" s="1" t="n">
         <v>5322</v>
@@ -12338,7 +12390,7 @@
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="O56" s="1" t="n">
         <f aca="false">AVERAGE(O41,O43,O47,O48,O54)</f>
@@ -12399,7 +12451,7 @@
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="O57" s="1" t="n">
         <f aca="false">AVERAGE(O38,O41,O43,O47,O48,O54,)</f>
@@ -12468,22 +12520,22 @@
       <c r="AG68" s="2"/>
       <c r="AH68" s="2"/>
       <c r="BC68" s="1" t="s">
-        <v>317</v>
+        <v>325</v>
       </c>
       <c r="BE68" s="1" t="s">
-        <v>282</v>
+        <v>290</v>
       </c>
       <c r="BF68" s="1" t="s">
-        <v>318</v>
+        <v>326</v>
       </c>
       <c r="BG68" s="1" t="s">
-        <v>319</v>
+        <v>327</v>
       </c>
       <c r="BI68" s="12" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="BK68" s="11" t="s">
-        <v>321</v>
+        <v>329</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12492,7 +12544,7 @@
       <c r="AG69" s="2"/>
       <c r="AH69" s="2"/>
       <c r="BC69" s="1" t="s">
-        <v>322</v>
+        <v>330</v>
       </c>
       <c r="BE69" s="19" t="n">
         <v>136.18</v>
@@ -12526,7 +12578,7 @@
       <c r="AG71" s="2"/>
       <c r="AH71" s="2"/>
       <c r="BC71" s="1" t="s">
-        <v>323</v>
+        <v>331</v>
       </c>
       <c r="BE71" s="19" t="n">
         <v>93180.82</v>
@@ -12546,19 +12598,19 @@
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Y72" s="1" t="s">
-        <v>317</v>
+        <v>325</v>
       </c>
       <c r="AA72" s="1" t="s">
         <v>138</v>
       </c>
       <c r="AB72" s="1" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
       <c r="AC72" s="1" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
       <c r="AD72" s="1" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="AF72" s="2"/>
       <c r="AG72" s="2"/>
@@ -12566,7 +12618,7 @@
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Y73" s="1" t="s">
-        <v>322</v>
+        <v>330</v>
       </c>
       <c r="AA73" s="19" t="n">
         <v>341.28</v>
@@ -12597,7 +12649,7 @@
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Y75" s="1" t="s">
-        <v>323</v>
+        <v>331</v>
       </c>
       <c r="AA75" s="19" t="n">
         <v>112691.32</v>
@@ -12642,369 +12694,369 @@
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>324</v>
+        <v>332</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>326</v>
+        <v>334</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="2" t="s">
-        <v>327</v>
+        <v>335</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>328</v>
+        <v>336</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C7" s="2" t="s">
-        <v>329</v>
+        <v>337</v>
       </c>
       <c r="P7" s="2" t="s">
-        <v>329</v>
+        <v>337</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C8" s="2" t="s">
-        <v>330</v>
+        <v>338</v>
       </c>
       <c r="P8" s="2" t="s">
-        <v>331</v>
+        <v>339</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D9" s="2" t="s">
-        <v>332</v>
+        <v>340</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E10" s="2" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
       <c r="R10" s="2" t="s">
-        <v>336</v>
+        <v>344</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E11" s="2" t="s">
-        <v>336</v>
+        <v>344</v>
       </c>
       <c r="S11" s="2" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="W11" s="2" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F12" s="2" t="s">
-        <v>337</v>
+        <v>345</v>
       </c>
       <c r="S12" s="2" t="s">
-        <v>337</v>
+        <v>345</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G13" s="2" t="s">
-        <v>338</v>
+        <v>346</v>
       </c>
       <c r="T13" s="2" t="s">
-        <v>339</v>
+        <v>347</v>
       </c>
       <c r="W13" s="2" t="s">
-        <v>340</v>
+        <v>348</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F14" s="2" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="S14" s="2" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F15" s="2" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="S15" s="2" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G16" s="2" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="T16" s="2" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G17" s="2" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="T17" s="2" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F18" s="2" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
       <c r="S18" s="2" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G19" s="2" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="T19" s="2" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E20" s="2" t="s">
-        <v>347</v>
+        <v>355</v>
       </c>
       <c r="R20" s="2" t="s">
-        <v>347</v>
+        <v>355</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D21" s="2" t="s">
-        <v>348</v>
+        <v>356</v>
       </c>
       <c r="Q21" s="2" t="s">
-        <v>348</v>
+        <v>356</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E22" s="2" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
       <c r="R22" s="2" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E23" s="2" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
       <c r="R23" s="2" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E24" s="2" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
       <c r="R24" s="2" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D25" s="2" t="s">
-        <v>352</v>
+        <v>360</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>353</v>
+        <v>361</v>
       </c>
       <c r="Q25" s="2" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E26" s="2" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
       <c r="R26" s="2" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E27" s="2" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
       <c r="R27" s="2" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D28" s="2" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>355</v>
+        <v>363</v>
       </c>
       <c r="Q28" s="2" t="s">
-        <v>356</v>
+        <v>364</v>
       </c>
       <c r="Z28" s="2" t="s">
-        <v>357</v>
+        <v>365</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E29" s="2" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
       <c r="R29" s="2" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E30" s="2" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
       <c r="R30" s="2" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D31" s="2" t="s">
-        <v>358</v>
+        <v>366</v>
       </c>
       <c r="Q31" s="2" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D32" s="2" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="R32" s="2" t="s">
-        <v>361</v>
+        <v>369</v>
       </c>
       <c r="U32" s="2" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E33" s="2" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="R33" s="2" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="S34" s="2" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E35" s="48" t="s">
-        <v>365</v>
+      <c r="E35" s="51" t="s">
+        <v>373</v>
       </c>
       <c r="S35" s="2" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E36" s="2" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="Q36" s="2" t="s">
-        <v>367</v>
+        <v>375</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F37" s="2" t="s">
-        <v>368</v>
+        <v>376</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F38" s="2" t="s">
-        <v>369</v>
+        <v>377</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F39" s="2" t="s">
-        <v>370</v>
+        <v>378</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F40" s="2" t="s">
-        <v>371</v>
+        <v>379</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G41" s="2" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H42" s="2" t="s">
-        <v>373</v>
+        <v>381</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H43" s="2" t="s">
-        <v>374</v>
+        <v>382</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I44" s="2" t="s">
-        <v>375</v>
+        <v>383</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="J45" s="2" t="s">
-        <v>376</v>
+        <v>384</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F46" s="2" t="s">
-        <v>377</v>
+        <v>385</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G47" s="2" t="s">
-        <v>378</v>
+        <v>386</v>
       </c>
       <c r="L47" s="2" t="s">
-        <v>379</v>
+        <v>387</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G48" s="2" t="s">
-        <v>374</v>
+        <v>382</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H49" s="2" t="s">
-        <v>375</v>
+        <v>383</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I50" s="2" t="s">
-        <v>376</v>
+        <v>384</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D52" s="2" t="s">
-        <v>380</v>
+        <v>388</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E53" s="2" t="s">
-        <v>381</v>
+        <v>389</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D54" s="2" t="s">
-        <v>347</v>
+        <v>355</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add dao only inconsistent script
</commit_message>
<xml_diff>
--- a/a_summary_comparison.xlsx
+++ b/a_summary_comparison.xlsx
@@ -34,13 +34,13 @@
     <t xml:space="preserve">NBS/NBB WITH NON MONO CLB &lt;C* miscount</t>
   </si>
   <si>
-    <t xml:space="preserve">19-30-57</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NBS/NBB MONOTONIC CLB + HOG2 Optimizations (SAME WITH or WITHOUT selFonUSet) 14-02-52 + 23-56-57 + 10-53-29/04-39-38 + 19-30-57 + 03-13-21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Single Dir Single (First) Node verF – 10-53-29 + 03-13-21</t>
+    <t xml:space="preserve">19-30-57+ 08-48-52</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NBS/NBB MONOTONIC CLB + HOG2 Optimizations (SAME WITH or WITHOUT selFonUSet) 14-02-52 + 23-56-57 + 10-53-29/04-39-38 + 19-30-57 + 03-13-21+ 08-48-52</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Single Dir Single (First) Node verF – 10-53-29 + 03-13-21 + 08-48-52</t>
   </si>
   <si>
     <t xml:space="preserve">16-27-29 +10-25-57 NonMono CLB, No HOG2 Opts</t>
@@ -58,28 +58,10 @@
     <t xml:space="preserve">MOST CONNECTED MONO CLB, HOG2 OPT, NO selFonUSet 14-02-52 + 23-58-57 + 10-53-29/04-39-38 + 01-03-41 + 03-13-21 + 02-03-56 + 20-28-41 + 05-32-21</t>
   </si>
   <si>
-    <t xml:space="preserve">SmallestG MONO CLG, HOG2 OPT, NO selFonUSet 14-02-52 + 23-58-57+ 10-53-29/04-39-38 + 01-03-41 + 03-13-21 + 20-30-47 + 05-34-32</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">SmallestGF</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> MONO CLG, HOG2 OPT, NO selFonUSet  14-02-52 + 23-58-57+ 10-53-29/04-39-38 + 01-03-41 + 03-13-21 + 20-30-47 + 05-34-32</t>
-    </r>
+    <t xml:space="preserve">SmallestG MONO CLG, HOG2 OPT, NO selFonUSet 14-02-52 + 23-58-57+ 10-53-29/04-39-38 + 01-03-41 + 03-13-21 + 20-30-47 + 05-34-32 + 08-48-52</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SmallestGF MONO CLG, HOG2 OPT, NO selFonUSet  14-02-52 + 23-58-57+ 10-53-29/04-39-38 + 01-03-41 + 03-13-21 + 20-30-47 + 05-34-32 + 08-48-52</t>
   </si>
   <si>
     <t xml:space="preserve">GBFHS F MONO CLG, HOG2 OPT, NO selFonUSet 04-49-55 + 10-35-42 + 23-49-57 + 10-53-29/04-39-38 + 01-03-41 + 03-13-21 + 02-03-56</t>
@@ -1542,11 +1524,15 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="20" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="20" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="20" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="20" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1554,15 +1540,11 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="20" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="20" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="2" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="20" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1598,7 +1580,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="10" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="21" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="9" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1606,15 +1592,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="9" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="9" xfId="21" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="21" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="10" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2793,7 +2775,7 @@
       <c r="AO4" s="6" t="s">
         <v>226</v>
       </c>
-      <c r="AW4" s="6"/>
+      <c r="AW4" s="13"/>
       <c r="AX4" s="6" t="s">
         <v>227</v>
       </c>
@@ -2803,26 +2785,26 @@
       <c r="BD4" s="8" t="s">
         <v>229</v>
       </c>
-      <c r="BE4" s="8"/>
+      <c r="BE4" s="14"/>
       <c r="BF4" s="6" t="s">
         <v>230</v>
       </c>
-      <c r="BG4" s="6"/>
+      <c r="BG4" s="13"/>
       <c r="BH4" s="6" t="s">
         <v>231</v>
       </c>
-      <c r="BI4" s="6"/>
+      <c r="BI4" s="13"/>
       <c r="BJ4" s="6" t="s">
         <v>232</v>
       </c>
       <c r="BT4" s="6" t="s">
         <v>233</v>
       </c>
-      <c r="BU4" s="13"/>
+      <c r="BU4" s="15"/>
       <c r="BV4" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="BW4" s="14" t="s">
+      <c r="BW4" s="6" t="s">
         <v>234</v>
       </c>
       <c r="BX4" s="6" t="s">
@@ -2831,14 +2813,14 @@
       <c r="BY4" s="6" t="s">
         <v>236</v>
       </c>
-      <c r="BZ4" s="13"/>
+      <c r="BZ4" s="15"/>
       <c r="CA4" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="CB4" s="14" t="s">
+      <c r="CB4" s="6" t="s">
         <v>237</v>
       </c>
-      <c r="CC4" s="15" t="s">
+      <c r="CC4" s="16" t="s">
         <v>238</v>
       </c>
       <c r="CE4" s="6" t="s">
@@ -2848,22 +2830,22 @@
       <c r="CL4" s="6" t="s">
         <v>239</v>
       </c>
-      <c r="CM4" s="13"/>
+      <c r="CM4" s="15"/>
       <c r="CN4" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="CO4" s="16"/>
+      <c r="CO4" s="17"/>
       <c r="CP4" s="8" t="s">
         <v>240</v>
       </c>
       <c r="CS4" s="6" t="s">
         <v>241</v>
       </c>
-      <c r="CT4" s="13"/>
+      <c r="CT4" s="15"/>
       <c r="CU4" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="CV4" s="16" t="s">
+      <c r="CV4" s="17" t="s">
         <v>242</v>
       </c>
       <c r="CW4" s="10" t="s">
@@ -2872,38 +2854,38 @@
       <c r="DB4" s="6" t="s">
         <v>244</v>
       </c>
-      <c r="DC4" s="6"/>
+      <c r="DC4" s="13"/>
       <c r="DD4" s="6" t="s">
         <v>194</v>
       </c>
-      <c r="DF4" s="16" t="s">
+      <c r="DF4" s="17" t="s">
         <v>245</v>
       </c>
-      <c r="DG4" s="17" t="s">
+      <c r="DG4" s="18" t="s">
         <v>246</v>
       </c>
       <c r="DI4" s="6" t="s">
         <v>247</v>
       </c>
-      <c r="DJ4" s="6"/>
+      <c r="DJ4" s="13"/>
       <c r="DK4" s="6" t="s">
         <v>199</v>
       </c>
-      <c r="DL4" s="14" t="s">
+      <c r="DL4" s="6" t="s">
         <v>248</v>
       </c>
-      <c r="DM4" s="15" t="s">
+      <c r="DM4" s="16" t="s">
         <v>249</v>
       </c>
       <c r="DQ4" s="6" t="s">
         <v>250</v>
       </c>
-      <c r="DR4" s="18"/>
+      <c r="DR4" s="17"/>
       <c r="DS4" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="DT4" s="13"/>
-      <c r="DU4" s="13"/>
+      <c r="DT4" s="15"/>
+      <c r="DU4" s="15"/>
       <c r="DV4" s="6" t="s">
         <v>251</v>
       </c>
@@ -2925,24 +2907,24 @@
       </c>
       <c r="U5" s="20"/>
       <c r="V5" s="20"/>
-      <c r="W5" s="18"/>
+      <c r="W5" s="17"/>
       <c r="X5" s="20"/>
       <c r="Y5" s="20"/>
       <c r="Z5" s="20"/>
       <c r="AA5" s="20"/>
       <c r="AB5" s="20"/>
       <c r="AC5" s="20"/>
-      <c r="AD5" s="13"/>
+      <c r="AD5" s="15"/>
       <c r="AE5" s="20"/>
       <c r="AF5" s="20"/>
       <c r="AG5" s="20"/>
       <c r="AH5" s="20"/>
       <c r="AI5" s="20"/>
       <c r="AJ5" s="20"/>
-      <c r="AK5" s="13"/>
+      <c r="AK5" s="15"/>
       <c r="AL5" s="20"/>
       <c r="AM5" s="20"/>
-      <c r="AN5" s="13"/>
+      <c r="AN5" s="15"/>
       <c r="AO5" s="20"/>
       <c r="AP5" s="20"/>
       <c r="AQ5" s="20"/>
@@ -2955,25 +2937,26 @@
       <c r="AU5" s="19" t="n">
         <v>5229761</v>
       </c>
-      <c r="BD5" s="6"/>
+      <c r="AX5" s="13"/>
+      <c r="BD5" s="13"/>
       <c r="BE5" s="6"/>
-      <c r="BF5" s="6"/>
-      <c r="BH5" s="6"/>
+      <c r="BF5" s="13"/>
+      <c r="BH5" s="13"/>
       <c r="BJ5" s="6"/>
-      <c r="BT5" s="13"/>
+      <c r="BT5" s="15"/>
       <c r="BV5" s="6"/>
-      <c r="BY5" s="13"/>
+      <c r="BY5" s="15"/>
       <c r="BZ5" s="2"/>
       <c r="CA5" s="6"/>
-      <c r="CL5" s="13"/>
+      <c r="CL5" s="15"/>
       <c r="CN5" s="6"/>
-      <c r="CS5" s="13"/>
+      <c r="CS5" s="15"/>
       <c r="CU5" s="6"/>
-      <c r="DB5" s="6"/>
+      <c r="DB5" s="13"/>
       <c r="DD5" s="6"/>
-      <c r="DI5" s="6"/>
+      <c r="DI5" s="13"/>
       <c r="DK5" s="6"/>
-      <c r="DQ5" s="13"/>
+      <c r="DQ5" s="15"/>
       <c r="DS5" s="6"/>
       <c r="DV5" s="6"/>
       <c r="DW5" s="6"/>
@@ -3263,15 +3246,32 @@
       <c r="AS7" s="19"/>
       <c r="AT7" s="19"/>
       <c r="AU7" s="19"/>
-      <c r="AX7" s="22"/>
+      <c r="AW7" s="27" t="n">
+        <v>32300299.42</v>
+      </c>
+      <c r="AX7" s="27" t="n">
+        <v>55141389.33</v>
+      </c>
       <c r="AY7" s="2"/>
       <c r="BA7" s="22"/>
-      <c r="BD7" s="23"/>
-      <c r="BE7" s="23"/>
-      <c r="BF7" s="22"/>
-      <c r="BG7" s="22"/>
-      <c r="BH7" s="22"/>
-      <c r="BI7" s="22"/>
+      <c r="BD7" s="27" t="n">
+        <v>48951315.87</v>
+      </c>
+      <c r="BE7" s="28" t="n">
+        <v>31361982.29</v>
+      </c>
+      <c r="BF7" s="27" t="n">
+        <v>51377355.29</v>
+      </c>
+      <c r="BG7" s="27" t="n">
+        <v>45033064.06</v>
+      </c>
+      <c r="BH7" s="27" t="n">
+        <v>51472715.72</v>
+      </c>
+      <c r="BI7" s="27" t="n">
+        <v>36032686.19</v>
+      </c>
       <c r="BJ7" s="22"/>
       <c r="BL7" s="20"/>
       <c r="BT7" s="21" t="n">
@@ -3281,7 +3281,7 @@
         <v>31617423.59</v>
       </c>
       <c r="BV7" s="22"/>
-      <c r="BW7" s="27" t="n">
+      <c r="BW7" s="26" t="n">
         <v>51265832.89</v>
       </c>
       <c r="BX7" s="26" t="n">
@@ -3294,10 +3294,10 @@
         <v>31777108.45</v>
       </c>
       <c r="CA7" s="22"/>
-      <c r="CB7" s="27" t="n">
+      <c r="CB7" s="26" t="n">
         <v>51232645.8</v>
       </c>
-      <c r="CC7" s="28" t="n">
+      <c r="CC7" s="29" t="n">
         <v>35748456.86</v>
       </c>
       <c r="CL7" s="21" t="n">
@@ -3307,7 +3307,7 @@
         <v>31066159.83</v>
       </c>
       <c r="CN7" s="22"/>
-      <c r="CO7" s="29" t="n">
+      <c r="CO7" s="25" t="n">
         <v>51976301.26</v>
       </c>
       <c r="CP7" s="25" t="n">
@@ -3320,28 +3320,36 @@
         <v>31566025.49</v>
       </c>
       <c r="CU7" s="22"/>
-      <c r="CV7" s="29" t="n">
+      <c r="CV7" s="25" t="n">
         <v>51192264.68</v>
       </c>
       <c r="CW7" s="30" t="n">
         <v>35683845.24</v>
       </c>
-      <c r="DB7" s="22"/>
-      <c r="DC7" s="22"/>
+      <c r="DB7" s="27" t="n">
+        <v>62472274.99</v>
+      </c>
+      <c r="DC7" s="27" t="n">
+        <v>33654856.02</v>
+      </c>
       <c r="DD7" s="22"/>
-      <c r="DF7" s="29" t="n">
+      <c r="DF7" s="25" t="n">
         <v>51289186.25</v>
       </c>
       <c r="DG7" s="30" t="n">
         <v>35739254.71</v>
       </c>
-      <c r="DI7" s="24"/>
-      <c r="DJ7" s="24"/>
+      <c r="DI7" s="31" t="n">
+        <v>69235465.82</v>
+      </c>
+      <c r="DJ7" s="27" t="n">
+        <v>42853564.69</v>
+      </c>
       <c r="DK7" s="22"/>
-      <c r="DL7" s="27" t="n">
+      <c r="DL7" s="26" t="n">
         <v>51052924.65</v>
       </c>
-      <c r="DM7" s="28" t="n">
+      <c r="DM7" s="29" t="n">
         <v>35829574.04</v>
       </c>
       <c r="DQ7" s="21" t="n">
@@ -4392,20 +4400,32 @@
       <c r="AW14" s="21" t="n">
         <v>3190.88</v>
       </c>
-      <c r="AX14" s="21" t="n">
-        <v>92952.98</v>
+      <c r="AX14" s="27" t="n">
+        <v>93741.04</v>
       </c>
       <c r="AY14" s="19"/>
       <c r="AZ14" s="25"/>
       <c r="BA14" s="23"/>
       <c r="BB14" s="23"/>
       <c r="BC14" s="23"/>
-      <c r="BD14" s="19"/>
-      <c r="BE14" s="19"/>
-      <c r="BF14" s="19"/>
-      <c r="BG14" s="19"/>
-      <c r="BH14" s="19"/>
-      <c r="BI14" s="19"/>
+      <c r="BD14" s="27" t="n">
+        <v>88083.5</v>
+      </c>
+      <c r="BE14" s="27" t="n">
+        <v>3157.68</v>
+      </c>
+      <c r="BF14" s="27" t="n">
+        <v>97583.44</v>
+      </c>
+      <c r="BG14" s="27" t="n">
+        <v>3203.02</v>
+      </c>
+      <c r="BH14" s="27" t="n">
+        <v>99196.2</v>
+      </c>
+      <c r="BI14" s="27" t="n">
+        <v>3295.62</v>
+      </c>
       <c r="BJ14" s="19"/>
       <c r="BK14" s="23"/>
       <c r="BL14" s="24"/>
@@ -4423,7 +4443,7 @@
         <v>2552.32</v>
       </c>
       <c r="BV14" s="19"/>
-      <c r="BW14" s="31" t="n">
+      <c r="BW14" s="21" t="n">
         <v>97583.44</v>
       </c>
       <c r="BX14" s="21" t="n">
@@ -4436,7 +4456,7 @@
         <v>2543.44</v>
       </c>
       <c r="CA14" s="19"/>
-      <c r="CB14" s="31" t="n">
+      <c r="CB14" s="21" t="n">
         <v>97583.44</v>
       </c>
       <c r="CC14" s="32" t="n">
@@ -4459,7 +4479,7 @@
       <c r="CN14" s="21" t="n">
         <v>110385.66</v>
       </c>
-      <c r="CO14" s="31" t="n">
+      <c r="CO14" s="21" t="n">
         <v>77149.22</v>
       </c>
       <c r="CP14" s="21" t="n">
@@ -4476,7 +4496,7 @@
       <c r="CU14" s="21" t="n">
         <v>78729.08</v>
       </c>
-      <c r="CV14" s="31" t="n">
+      <c r="CV14" s="21" t="n">
         <v>97583.44</v>
       </c>
       <c r="CW14" s="32" t="n">
@@ -4486,20 +4506,28 @@
       <c r="CY14" s="23"/>
       <c r="CZ14" s="19"/>
       <c r="DA14" s="26"/>
-      <c r="DB14" s="23"/>
-      <c r="DC14" s="23"/>
+      <c r="DB14" s="27" t="n">
+        <v>79594.06</v>
+      </c>
+      <c r="DC14" s="27" t="n">
+        <v>2607.6</v>
+      </c>
       <c r="DD14" s="19"/>
-      <c r="DF14" s="31" t="n">
+      <c r="DF14" s="21" t="n">
         <v>97583.44</v>
       </c>
       <c r="DG14" s="32" t="n">
         <v>3534.9</v>
       </c>
       <c r="DH14" s="24"/>
-      <c r="DI14" s="25"/>
-      <c r="DJ14" s="25"/>
+      <c r="DI14" s="27" t="n">
+        <v>90855.52</v>
+      </c>
+      <c r="DJ14" s="27" t="n">
+        <v>2599.28</v>
+      </c>
       <c r="DK14" s="19"/>
-      <c r="DL14" s="31" t="n">
+      <c r="DL14" s="21" t="n">
         <v>97583.44</v>
       </c>
       <c r="DM14" s="32" t="n">
@@ -4550,6 +4578,8 @@
       <c r="A16" s="1" t="s">
         <v>260</v>
       </c>
+      <c r="BH16" s="27"/>
+      <c r="DI16" s="27"/>
       <c r="DO16" s="2"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4617,18 +4647,24 @@
         <v>675705.86</v>
       </c>
       <c r="BC17" s="21"/>
-      <c r="BD17" s="23" t="n">
+      <c r="BD17" s="27" t="n">
         <v>675108.9</v>
       </c>
-      <c r="BE17" s="23"/>
+      <c r="BE17" s="27" t="n">
+        <v>676377.66</v>
+      </c>
       <c r="BF17" s="21" t="n">
         <v>666626.74</v>
       </c>
-      <c r="BG17" s="21"/>
+      <c r="BG17" s="27" t="n">
+        <v>668932.26</v>
+      </c>
       <c r="BH17" s="22" t="n">
         <v>675760.32</v>
       </c>
-      <c r="BI17" s="22"/>
+      <c r="BI17" s="27" t="n">
+        <v>677524.82</v>
+      </c>
       <c r="BJ17" s="22" t="n">
         <v>669452.3</v>
       </c>
@@ -4720,7 +4756,9 @@
       <c r="DB17" s="21" t="n">
         <v>652385.48</v>
       </c>
-      <c r="DC17" s="21"/>
+      <c r="DC17" s="27" t="n">
+        <v>655946.28</v>
+      </c>
       <c r="DD17" s="22" t="n">
         <v>652385.48</v>
       </c>
@@ -4729,7 +4767,9 @@
       <c r="DI17" s="22" t="n">
         <v>651572.04</v>
       </c>
-      <c r="DJ17" s="22"/>
+      <c r="DJ17" s="27" t="n">
+        <v>650178.52</v>
+      </c>
       <c r="DK17" s="21" t="n">
         <v>4302122.84</v>
       </c>
@@ -5549,7 +5589,7 @@
         <v>219076.92</v>
       </c>
       <c r="BV21" s="2"/>
-      <c r="BW21" s="31" t="n">
+      <c r="BW21" s="21" t="n">
         <v>864030.18</v>
       </c>
       <c r="BX21" s="21" t="n">
@@ -5562,7 +5602,7 @@
         <v>213123.84</v>
       </c>
       <c r="CA21" s="2"/>
-      <c r="CB21" s="31" t="n">
+      <c r="CB21" s="21" t="n">
         <v>864030.18</v>
       </c>
       <c r="CC21" s="32" t="n">
@@ -5583,7 +5623,7 @@
         <v>267819.92</v>
       </c>
       <c r="CN21" s="2"/>
-      <c r="CO21" s="31" t="n">
+      <c r="CO21" s="21" t="n">
         <v>785705.64</v>
       </c>
       <c r="CP21" s="21" t="n">
@@ -5596,7 +5636,7 @@
         <v>219100.06</v>
       </c>
       <c r="CU21" s="2"/>
-      <c r="CV21" s="31" t="n">
+      <c r="CV21" s="21" t="n">
         <v>864030.18</v>
       </c>
       <c r="CW21" s="32" t="n">
@@ -5612,7 +5652,7 @@
         <v>218965.4</v>
       </c>
       <c r="DD21" s="2"/>
-      <c r="DF21" s="31" t="n">
+      <c r="DF21" s="21" t="n">
         <v>864030.18</v>
       </c>
       <c r="DG21" s="32" t="n">
@@ -5625,7 +5665,7 @@
         <v>452466.44</v>
       </c>
       <c r="DK21" s="2"/>
-      <c r="DL21" s="31" t="n">
+      <c r="DL21" s="21" t="n">
         <v>864030.18</v>
       </c>
       <c r="DM21" s="32" t="n">
@@ -5758,7 +5798,7 @@
         <v>700648.08</v>
       </c>
       <c r="BV22" s="2"/>
-      <c r="BW22" s="27" t="n">
+      <c r="BW22" s="26" t="n">
         <v>691182.52</v>
       </c>
       <c r="BX22" s="26" t="n">
@@ -5771,10 +5811,10 @@
         <v>701793.04</v>
       </c>
       <c r="CA22" s="2"/>
-      <c r="CB22" s="27" t="n">
+      <c r="CB22" s="26" t="n">
         <v>691182.52</v>
       </c>
-      <c r="CC22" s="28" t="n">
+      <c r="CC22" s="29" t="n">
         <v>680903.3</v>
       </c>
       <c r="CD22" s="24"/>
@@ -5792,7 +5832,7 @@
         <v>664150.56</v>
       </c>
       <c r="CN22" s="2"/>
-      <c r="CO22" s="29" t="n">
+      <c r="CO22" s="25" t="n">
         <v>679944.1</v>
       </c>
       <c r="CP22" s="25" t="n">
@@ -5805,7 +5845,7 @@
         <v>700649.46</v>
       </c>
       <c r="CU22" s="2"/>
-      <c r="CV22" s="29" t="n">
+      <c r="CV22" s="25" t="n">
         <v>691182.52</v>
       </c>
       <c r="CW22" s="30" t="n">
@@ -5821,7 +5861,7 @@
         <v>701507.72</v>
       </c>
       <c r="DD22" s="2"/>
-      <c r="DF22" s="29" t="n">
+      <c r="DF22" s="25" t="n">
         <v>691182.52</v>
       </c>
       <c r="DG22" s="30" t="n">
@@ -5834,10 +5874,10 @@
         <v>700405.84</v>
       </c>
       <c r="DK22" s="2"/>
-      <c r="DL22" s="27" t="n">
+      <c r="DL22" s="26" t="n">
         <v>691182.52</v>
       </c>
-      <c r="DM22" s="28" t="n">
+      <c r="DM22" s="29" t="n">
         <v>680903.3</v>
       </c>
       <c r="DO22" s="24"/>
@@ -6256,7 +6296,7 @@
       <c r="BU29" s="21" t="n">
         <v>5862.43251825977</v>
       </c>
-      <c r="BW29" s="27" t="n">
+      <c r="BW29" s="26" t="n">
         <v>46193.2429342649</v>
       </c>
       <c r="BX29" s="26" t="n">
@@ -6268,10 +6308,10 @@
       <c r="BZ29" s="21" t="n">
         <v>5850.13718640838</v>
       </c>
-      <c r="CB29" s="27" t="n">
+      <c r="CB29" s="26" t="n">
         <v>46193.2429342649</v>
       </c>
-      <c r="CC29" s="28" t="n">
+      <c r="CC29" s="29" t="n">
         <v>8041.30930454112</v>
       </c>
       <c r="CL29" s="21" t="n">
@@ -6280,7 +6320,7 @@
       <c r="CM29" s="21" t="n">
         <v>6514.37313432836</v>
       </c>
-      <c r="CO29" s="29" t="n">
+      <c r="CO29" s="25" t="n">
         <v>35644.430612893</v>
       </c>
       <c r="CP29" s="25" t="n">
@@ -6292,22 +6332,22 @@
       <c r="CT29" s="21" t="n">
         <v>5841.05080978088</v>
       </c>
-      <c r="CV29" s="29" t="n">
+      <c r="CV29" s="25" t="n">
         <v>46193.2429342649</v>
       </c>
       <c r="CW29" s="30" t="n">
         <v>8041.30930454112</v>
       </c>
-      <c r="DF29" s="29" t="n">
+      <c r="DF29" s="25" t="n">
         <v>46193.2429342649</v>
       </c>
       <c r="DG29" s="30" t="n">
         <v>8041.30930454112</v>
       </c>
-      <c r="DL29" s="27" t="n">
+      <c r="DL29" s="26" t="n">
         <v>46193.2429342649</v>
       </c>
-      <c r="DM29" s="28" t="n">
+      <c r="DM29" s="29" t="n">
         <v>8041.30930454112</v>
       </c>
       <c r="DO29" s="2"/>
@@ -6877,14 +6917,31 @@
       <c r="AS46" s="35"/>
       <c r="AT46" s="35"/>
       <c r="AU46" s="35"/>
-      <c r="AX46" s="21"/>
+      <c r="AW46" s="27" t="n">
+        <v>32198352.4</v>
+      </c>
+      <c r="AX46" s="27" t="n">
+        <v>55102989.2</v>
+      </c>
       <c r="BA46" s="21"/>
-      <c r="BD46" s="25"/>
-      <c r="BE46" s="25"/>
-      <c r="BF46" s="21"/>
-      <c r="BG46" s="21"/>
-      <c r="BH46" s="21"/>
-      <c r="BI46" s="21"/>
+      <c r="BD46" s="27" t="n">
+        <v>48880460.36</v>
+      </c>
+      <c r="BE46" s="28" t="n">
+        <v>31084273.89</v>
+      </c>
+      <c r="BF46" s="27" t="n">
+        <v>50978864.83</v>
+      </c>
+      <c r="BG46" s="27" t="n">
+        <v>44811738.43</v>
+      </c>
+      <c r="BH46" s="27" t="n">
+        <v>51368391.37</v>
+      </c>
+      <c r="BI46" s="27" t="n">
+        <v>35745851.67</v>
+      </c>
       <c r="BJ46" s="21"/>
       <c r="BL46" s="20"/>
       <c r="BT46" s="21" t="n">
@@ -6894,7 +6951,7 @@
         <v>31320394.4</v>
       </c>
       <c r="BV46" s="21"/>
-      <c r="BW46" s="27" t="n">
+      <c r="BW46" s="26" t="n">
         <v>50887944.49</v>
       </c>
       <c r="BX46" s="26" t="n">
@@ -6907,10 +6964,10 @@
         <v>31444760.94</v>
       </c>
       <c r="CA46" s="21"/>
-      <c r="CB46" s="27" t="n">
+      <c r="CB46" s="26" t="n">
         <v>50889522.5</v>
       </c>
-      <c r="CC46" s="28" t="n">
+      <c r="CC46" s="29" t="n">
         <v>35508088.94</v>
       </c>
       <c r="CL46" s="21" t="n">
@@ -6920,7 +6977,7 @@
         <v>29387631.87</v>
       </c>
       <c r="CN46" s="21"/>
-      <c r="CO46" s="29" t="n">
+      <c r="CO46" s="25" t="n">
         <v>47520623.52</v>
       </c>
       <c r="CP46" s="25" t="n">
@@ -6933,28 +6990,36 @@
         <v>31315234.05</v>
       </c>
       <c r="CU46" s="21"/>
-      <c r="CV46" s="29" t="n">
+      <c r="CV46" s="25" t="n">
         <v>50887883.09</v>
       </c>
       <c r="CW46" s="30" t="n">
         <v>35510968.78</v>
       </c>
-      <c r="DB46" s="21"/>
-      <c r="DC46" s="21"/>
+      <c r="DB46" s="27" t="n">
+        <v>60608583.49</v>
+      </c>
+      <c r="DC46" s="27" t="n">
+        <v>33461481.24</v>
+      </c>
       <c r="DD46" s="21"/>
-      <c r="DF46" s="29" t="n">
+      <c r="DF46" s="25" t="n">
         <v>50887897.01</v>
       </c>
       <c r="DG46" s="30" t="n">
         <v>35508467.79</v>
       </c>
-      <c r="DI46" s="26"/>
-      <c r="DJ46" s="26"/>
+      <c r="DI46" s="31" t="n">
+        <v>69188574.16</v>
+      </c>
+      <c r="DJ46" s="27" t="n">
+        <v>42646181.29</v>
+      </c>
       <c r="DK46" s="21"/>
-      <c r="DL46" s="27" t="n">
+      <c r="DL46" s="26" t="n">
         <v>50983233.34</v>
       </c>
-      <c r="DM46" s="28" t="n">
+      <c r="DM46" s="29" t="n">
         <v>35569628.97</v>
       </c>
       <c r="DO46" s="2"/>
@@ -7925,20 +7990,32 @@
       <c r="AW53" s="37" t="n">
         <v>1780.36</v>
       </c>
-      <c r="AX53" s="37" t="n">
-        <v>64724.76</v>
+      <c r="AX53" s="27" t="n">
+        <v>64759.4</v>
       </c>
       <c r="AY53" s="20"/>
       <c r="AZ53" s="25"/>
       <c r="BA53" s="25"/>
       <c r="BB53" s="25"/>
       <c r="BC53" s="25"/>
-      <c r="BD53" s="35"/>
-      <c r="BE53" s="35"/>
-      <c r="BF53" s="35"/>
-      <c r="BG53" s="35"/>
-      <c r="BH53" s="35"/>
-      <c r="BI53" s="35"/>
+      <c r="BD53" s="27" t="n">
+        <v>61339.12</v>
+      </c>
+      <c r="BE53" s="27" t="n">
+        <v>1745.24</v>
+      </c>
+      <c r="BF53" s="27" t="n">
+        <v>60992.46</v>
+      </c>
+      <c r="BG53" s="27" t="n">
+        <v>1775.8</v>
+      </c>
+      <c r="BH53" s="27" t="n">
+        <v>59940.52</v>
+      </c>
+      <c r="BI53" s="27" t="n">
+        <v>1825.32</v>
+      </c>
       <c r="BJ53" s="35"/>
       <c r="BK53" s="25"/>
       <c r="BL53" s="38"/>
@@ -7956,7 +8033,7 @@
         <v>1482.4</v>
       </c>
       <c r="BV53" s="20"/>
-      <c r="BW53" s="31" t="n">
+      <c r="BW53" s="21" t="n">
         <v>60992.46</v>
       </c>
       <c r="BX53" s="21" t="n">
@@ -7969,7 +8046,7 @@
         <v>1466.44</v>
       </c>
       <c r="CA53" s="35"/>
-      <c r="CB53" s="31" t="n">
+      <c r="CB53" s="21" t="n">
         <v>60992.46</v>
       </c>
       <c r="CC53" s="32" t="n">
@@ -7992,7 +8069,7 @@
       <c r="CN53" s="37" t="n">
         <v>44688.26</v>
       </c>
-      <c r="CO53" s="31" t="n">
+      <c r="CO53" s="21" t="n">
         <v>55953.14</v>
       </c>
       <c r="CP53" s="21" t="n">
@@ -8009,7 +8086,7 @@
       <c r="CU53" s="37" t="n">
         <v>52187.04</v>
       </c>
-      <c r="CV53" s="31" t="n">
+      <c r="CV53" s="21" t="n">
         <v>60992.46</v>
       </c>
       <c r="CW53" s="32" t="n">
@@ -8019,20 +8096,28 @@
       <c r="CY53" s="36"/>
       <c r="CZ53" s="35"/>
       <c r="DA53" s="26"/>
-      <c r="DB53" s="25"/>
-      <c r="DC53" s="25"/>
+      <c r="DB53" s="27" t="n">
+        <v>51989.54</v>
+      </c>
+      <c r="DC53" s="27" t="n">
+        <v>1503.42</v>
+      </c>
       <c r="DD53" s="20"/>
-      <c r="DF53" s="31" t="n">
+      <c r="DF53" s="21" t="n">
         <v>60992.46</v>
       </c>
       <c r="DG53" s="32" t="n">
         <v>1775.4</v>
       </c>
       <c r="DH53" s="38"/>
-      <c r="DI53" s="36"/>
-      <c r="DJ53" s="36"/>
+      <c r="DI53" s="27" t="n">
+        <v>48451.08</v>
+      </c>
+      <c r="DJ53" s="27" t="n">
+        <v>1554.86</v>
+      </c>
       <c r="DK53" s="20"/>
-      <c r="DL53" s="31" t="n">
+      <c r="DL53" s="21" t="n">
         <v>60992.46</v>
       </c>
       <c r="DM53" s="32" t="n">
@@ -8157,15 +8242,21 @@
       <c r="BD56" s="36" t="n">
         <v>660993.9</v>
       </c>
-      <c r="BE56" s="36"/>
+      <c r="BE56" s="27" t="n">
+        <v>660978.4</v>
+      </c>
       <c r="BF56" s="37" t="n">
         <v>649770.12</v>
       </c>
-      <c r="BG56" s="37"/>
+      <c r="BG56" s="27" t="n">
+        <v>651367.52</v>
+      </c>
       <c r="BH56" s="37" t="n">
         <v>663178.46</v>
       </c>
-      <c r="BI56" s="37"/>
+      <c r="BI56" s="27" t="n">
+        <v>663175.52</v>
+      </c>
       <c r="BJ56" s="37" t="n">
         <v>663089.96</v>
       </c>
@@ -8259,7 +8350,9 @@
       <c r="DB56" s="21" t="n">
         <v>628142.9</v>
       </c>
-      <c r="DC56" s="21"/>
+      <c r="DC56" s="27" t="n">
+        <v>628120.02</v>
+      </c>
       <c r="DD56" s="37" t="n">
         <v>628142.9</v>
       </c>
@@ -8268,7 +8361,9 @@
       <c r="DI56" s="21" t="n">
         <v>639195.4</v>
       </c>
-      <c r="DJ56" s="21"/>
+      <c r="DJ56" s="27" t="n">
+        <v>644133.8</v>
+      </c>
       <c r="DK56" s="37" t="n">
         <v>4297524.02</v>
       </c>
@@ -9024,7 +9119,7 @@
         <v>219013.9</v>
       </c>
       <c r="BV60" s="2"/>
-      <c r="BW60" s="31" t="n">
+      <c r="BW60" s="21" t="n">
         <v>857506.12</v>
       </c>
       <c r="BX60" s="21" t="n">
@@ -9037,7 +9132,7 @@
         <v>212803.62</v>
       </c>
       <c r="CA60" s="2"/>
-      <c r="CB60" s="31" t="n">
+      <c r="CB60" s="21" t="n">
         <v>857506.12</v>
       </c>
       <c r="CC60" s="32" t="n">
@@ -9058,7 +9153,7 @@
         <v>267261.84</v>
       </c>
       <c r="CN60" s="2"/>
-      <c r="CO60" s="31" t="n">
+      <c r="CO60" s="21" t="n">
         <v>766251.24</v>
       </c>
       <c r="CP60" s="21" t="n">
@@ -9071,7 +9166,7 @@
         <v>219037.52</v>
       </c>
       <c r="CU60" s="2"/>
-      <c r="CV60" s="31" t="n">
+      <c r="CV60" s="21" t="n">
         <v>857506.12</v>
       </c>
       <c r="CW60" s="32" t="n">
@@ -9087,7 +9182,7 @@
         <v>218903.2</v>
       </c>
       <c r="DD60" s="2"/>
-      <c r="DF60" s="31" t="n">
+      <c r="DF60" s="21" t="n">
         <v>857506.12</v>
       </c>
       <c r="DG60" s="32" t="n">
@@ -9100,7 +9195,7 @@
         <v>452466.42</v>
       </c>
       <c r="DK60" s="2"/>
-      <c r="DL60" s="31" t="n">
+      <c r="DL60" s="21" t="n">
         <v>857506.12</v>
       </c>
       <c r="DM60" s="32" t="n">
@@ -9234,7 +9329,7 @@
         <v>672259.18</v>
       </c>
       <c r="BV61" s="2"/>
-      <c r="BW61" s="27" t="n">
+      <c r="BW61" s="26" t="n">
         <v>679771.56</v>
       </c>
       <c r="BX61" s="26" t="n">
@@ -9247,10 +9342,10 @@
         <v>675108.8</v>
       </c>
       <c r="CA61" s="2"/>
-      <c r="CB61" s="27" t="n">
+      <c r="CB61" s="26" t="n">
         <v>679771.56</v>
       </c>
-      <c r="CC61" s="28" t="n">
+      <c r="CC61" s="29" t="n">
         <v>657634.88</v>
       </c>
       <c r="CD61" s="26"/>
@@ -9268,7 +9363,7 @@
         <v>634996.82</v>
       </c>
       <c r="CN61" s="2"/>
-      <c r="CO61" s="29" t="n">
+      <c r="CO61" s="25" t="n">
         <v>667290.94</v>
       </c>
       <c r="CP61" s="25" t="n">
@@ -9281,7 +9376,7 @@
         <v>671967.04</v>
       </c>
       <c r="CU61" s="2"/>
-      <c r="CV61" s="29" t="n">
+      <c r="CV61" s="25" t="n">
         <v>679771.56</v>
       </c>
       <c r="CW61" s="30" t="n">
@@ -9297,7 +9392,7 @@
         <v>672930.84</v>
       </c>
       <c r="DD61" s="2"/>
-      <c r="DF61" s="29" t="n">
+      <c r="DF61" s="25" t="n">
         <v>679771.56</v>
       </c>
       <c r="DG61" s="30" t="n">
@@ -9310,10 +9405,10 @@
         <v>682476.76</v>
       </c>
       <c r="DK61" s="2"/>
-      <c r="DL61" s="27" t="n">
+      <c r="DL61" s="26" t="n">
         <v>679771.56</v>
       </c>
-      <c r="DM61" s="28" t="n">
+      <c r="DM61" s="29" t="n">
         <v>657634.88</v>
       </c>
       <c r="DO61" s="38"/>
@@ -9619,7 +9714,7 @@
       <c r="BU68" s="21" t="n">
         <v>5309.3569387107</v>
       </c>
-      <c r="BW68" s="27" t="n">
+      <c r="BW68" s="26" t="n">
         <v>44620.6024134646</v>
       </c>
       <c r="BX68" s="26" t="n">
@@ -9631,10 +9726,10 @@
       <c r="BZ68" s="21" t="n">
         <v>5297.03683709114</v>
       </c>
-      <c r="CB68" s="27" t="n">
+      <c r="CB68" s="26" t="n">
         <v>44620.6024134646</v>
       </c>
-      <c r="CC68" s="28" t="n">
+      <c r="CC68" s="29" t="n">
         <v>7499.07589711019</v>
       </c>
       <c r="CL68" s="21" t="n">
@@ -9643,7 +9738,7 @@
       <c r="CM68" s="21" t="n">
         <v>6148.27723086694</v>
       </c>
-      <c r="CO68" s="29" t="n">
+      <c r="CO68" s="25" t="n">
         <v>35070.1571927596</v>
       </c>
       <c r="CP68" s="25" t="n">
@@ -9655,22 +9750,22 @@
       <c r="CT68" s="21" t="n">
         <v>5288.7897745316</v>
       </c>
-      <c r="CV68" s="29" t="n">
+      <c r="CV68" s="25" t="n">
         <v>44620.6024134646</v>
       </c>
       <c r="CW68" s="30" t="n">
         <v>7499.07589711019</v>
       </c>
-      <c r="DF68" s="29" t="n">
+      <c r="DF68" s="25" t="n">
         <v>44620.6024134646</v>
       </c>
       <c r="DG68" s="30" t="n">
         <v>7499.07589711019</v>
       </c>
-      <c r="DL68" s="27" t="n">
+      <c r="DL68" s="26" t="n">
         <v>44620.6024134646</v>
       </c>
-      <c r="DM68" s="28" t="n">
+      <c r="DM68" s="29" t="n">
         <v>7499.07589711019</v>
       </c>
       <c r="DQ68" s="21" t="n">

</xml_diff>